<commit_message>
ACTUALIZACION DEL ARCHIVO EMPLEADOS
</commit_message>
<xml_diff>
--- a/CONCENTRADO_EMPLEADOS.xlsx
+++ b/CONCENTRADO_EMPLEADOS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4604c7d1701c1fd5/Desktop/bagira_agent/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4604c7d1701c1fd5/Desktop/BagheeraAgent/BageheeraAgent/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="11_11F15350D473D61EE10F68D7565DCE3A874760D9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56F50349-EA9C-4EFA-B825-3831A7C16439}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="11_11F15350D473D61EE10F68D7565DCE3A874760D9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D140A83F-CCB6-4131-AAE6-9DB3A81CE4D6}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="173">
   <si>
     <t>ID</t>
   </si>
@@ -527,6 +527,18 @@
   </si>
   <si>
     <t xml:space="preserve"> ROCHA BONILLA ARIANA ISABEL</t>
+  </si>
+  <si>
+    <t>MARTINEZ HERNANDEZ DANNA PAOLA</t>
+  </si>
+  <si>
+    <t>RUNNER</t>
+  </si>
+  <si>
+    <t>MAHD051009MTSRRNA8</t>
+  </si>
+  <si>
+    <t>C AQUILES SERDAN #202 COL AMPLIACION LAGUNA DE LA PUERTA</t>
   </si>
 </sst>
 </file>
@@ -534,7 +546,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -567,8 +579,8 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -871,11 +883,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K46"/>
+  <dimension ref="A1:K47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="36.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="18" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="70.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
@@ -1342,7 +1357,7 @@
       <c r="A15">
         <v>19.100000000000001</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" t="s">
         <v>54</v>
       </c>
       <c r="C15" t="s">
@@ -2414,6 +2429,41 @@
       </c>
       <c r="K46" t="s">
         <v>156</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A47">
+        <v>63</v>
+      </c>
+      <c r="B47" t="s">
+        <v>169</v>
+      </c>
+      <c r="C47" t="s">
+        <v>44</v>
+      </c>
+      <c r="D47" t="s">
+        <v>170</v>
+      </c>
+      <c r="E47" s="2">
+        <v>46095</v>
+      </c>
+      <c r="F47" t="s">
+        <v>20</v>
+      </c>
+      <c r="G47" s="2">
+        <v>46187</v>
+      </c>
+      <c r="H47" t="s">
+        <v>14</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J47" t="s">
+        <v>171</v>
+      </c>
+      <c r="K47" s="2" t="s">
+        <v>172</v>
       </c>
     </row>
   </sheetData>

</xml_diff>